<commit_message>
Documentation NAV Calculator et module fund-of-funds dans README
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E997E5-A300-4887-B820-928BACDACE70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1792F02A-8FFF-4A22-8EB2-02E21EE2E3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
     <sheet name="Liabilities" sheetId="2" r:id="rId2"/>
     <sheet name="NAV Calculation" sheetId="3" r:id="rId3"/>
+    <sheet name="Fund-of-Funds" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
   <si>
     <t>Asset Type</t>
   </si>
@@ -128,6 +129,36 @@
   </si>
   <si>
     <t>NAV per Share</t>
+  </si>
+  <si>
+    <t>Sous-fonds</t>
+  </si>
+  <si>
+    <t>Parts détenues</t>
+  </si>
+  <si>
+    <t>NAV par part du sous fonds</t>
+  </si>
+  <si>
+    <t>Frais du sous-fonds (annuel)</t>
+  </si>
+  <si>
+    <t>Sous-fonds A (obligations)</t>
+  </si>
+  <si>
+    <t>Sous-fonds B (actions US)</t>
+  </si>
+  <si>
+    <t>Sous-fonds C (actions émergentes)</t>
+  </si>
+  <si>
+    <t>Valeur de marché</t>
+  </si>
+  <si>
+    <t>Frais courus journaliers</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
@@ -162,7 +193,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -178,6 +209,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -206,11 +243,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -235,10 +273,19 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Pourcentage" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -835,4 +882,121 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBC3DFD7-3973-48BA-AFC4-B88EAA110AFA}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" customWidth="1"/>
+    <col min="5" max="5" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="3">
+        <v>500</v>
+      </c>
+      <c r="C2" s="3">
+        <v>105</v>
+      </c>
+      <c r="D2" s="16">
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="E2" s="3">
+        <f>+B2*C2</f>
+        <v>52500</v>
+      </c>
+      <c r="F2" s="3">
+        <f>+(E2*D2)/365</f>
+        <v>1.1506849315068493</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="3">
+        <v>300</v>
+      </c>
+      <c r="C3" s="3">
+        <v>210</v>
+      </c>
+      <c r="D3" s="16">
+        <v>1.2E-2</v>
+      </c>
+      <c r="E3" s="3">
+        <f t="shared" ref="E3:E4" si="0">+B3*C3</f>
+        <v>63000</v>
+      </c>
+      <c r="F3" s="3">
+        <f t="shared" ref="F3:F4" si="1">+(E3*D3)/365</f>
+        <v>2.0712328767123287</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="3">
+        <v>200</v>
+      </c>
+      <c r="C4" s="3">
+        <v>95</v>
+      </c>
+      <c r="D4" s="17">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="E4" s="3">
+        <f t="shared" si="0"/>
+        <v>19000</v>
+      </c>
+      <c r="F4" s="3">
+        <f t="shared" si="1"/>
+        <v>0.78082191780821919</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5">
+        <f>+SUM(E2:E4)</f>
+        <v>134500</v>
+      </c>
+      <c r="F5">
+        <f>+SUM(F2:F4)</f>
+        <v>4.0027397260273974</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Nettoyage fichier temporaire Excel + ajout .gitignore
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1792F02A-8FFF-4A22-8EB2-02E21EE2E3A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976C89CA-9081-4A9A-9F68-F739A5C95E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t>Asset Type</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Fund-of-Funds investment</t>
+  </si>
+  <si>
+    <t>Position consolidée 3 sous-fonds UCITS</t>
+  </si>
+  <si>
+    <t>Frais courus - Fund-of-Funds</t>
   </si>
 </sst>
 </file>
@@ -248,7 +257,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -281,6 +290,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -617,7 +636,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E07DA19-FCC4-447D-B132-7320A0C60E42}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.109375" bestFit="1" customWidth="1"/>
@@ -654,7 +673,7 @@
       <c r="D2" s="4">
         <v>650</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="22">
         <f>+D2*C2</f>
         <v>130000</v>
       </c>
@@ -672,7 +691,7 @@
       <c r="D3" s="4">
         <v>720</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="22">
         <f t="shared" ref="E3:E4" si="0">+D3*C3</f>
         <v>108000</v>
       </c>
@@ -690,7 +709,7 @@
       <c r="D4" s="4">
         <v>410</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="22">
         <f t="shared" si="0"/>
         <v>123000</v>
       </c>
@@ -704,7 +723,7 @@
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="6"/>
-      <c r="E5" s="6">
+      <c r="E5" s="21">
         <v>85000</v>
       </c>
     </row>
@@ -717,7 +736,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6"/>
-      <c r="E6" s="6">
+      <c r="E6" s="21">
         <v>3200</v>
       </c>
     </row>
@@ -730,20 +749,34 @@
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="6"/>
-      <c r="E7" s="6">
+      <c r="E7" s="21">
         <v>1150</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="21">
+        <f>+'Fund-of-Funds'!E5</f>
+        <v>134500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="10">
-        <f>+SUM(E2:E7)</f>
-        <v>450350</v>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="10">
+        <f>+SUM(E2:E8)</f>
+        <v>584850</v>
       </c>
     </row>
   </sheetData>
@@ -753,7 +786,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A23F0DBC-E8D0-4A44-A3D3-1DDCFD82E51B}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
@@ -790,8 +823,8 @@
         <v>22</v>
       </c>
       <c r="C3" s="4">
-        <f>+(Assets!E8*Liabilities!F3)/365</f>
-        <v>12.338356164383562</v>
+        <f>+(Assets!E9*Liabilities!F3)/365</f>
+        <v>16.023287671232875</v>
       </c>
       <c r="F3" s="7">
         <v>0.01</v>
@@ -809,17 +842,29 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="4">
+        <f>+'Fund-of-Funds'!F5</f>
+        <v>4.0027397260273974</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="9">
-        <f>+SUM(C2:C4)</f>
-        <v>4312.3383561643841</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C6" s="1"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="9">
+        <f>+SUM(C2:C5)</f>
+        <v>4320.0260273972599</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C7" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -840,8 +885,8 @@
         <v>24</v>
       </c>
       <c r="B1" s="12">
-        <f>+Assets!E8</f>
-        <v>450350</v>
+        <f>+Assets!E9</f>
+        <v>584850</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -849,8 +894,8 @@
         <v>25</v>
       </c>
       <c r="B2" s="12">
-        <f>+Liabilities!C5</f>
-        <v>4312.3383561643841</v>
+        <f>+Liabilities!C6</f>
+        <v>4320.0260273972599</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -859,7 +904,7 @@
       </c>
       <c r="B3" s="13">
         <f>+B1-B2</f>
-        <v>446037.6616438356</v>
+        <v>580529.97397260275</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -876,7 +921,7 @@
       </c>
       <c r="B5" s="15">
         <f>+B3/B4</f>
-        <v>99.561978045499018</v>
+        <v>129.58258347602739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Documentation étape 3 : journal; trial balance, NAV tie-out
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976C89CA-9081-4A9A-9F68-F739A5C95E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457DAB21-DA21-44E9-8C80-5FA1D9C46E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
     <sheet name="Liabilities" sheetId="2" r:id="rId2"/>
     <sheet name="NAV Calculation" sheetId="3" r:id="rId3"/>
     <sheet name="Fund-of-Funds" sheetId="4" r:id="rId4"/>
+    <sheet name="Transaction Journal" sheetId="5" r:id="rId5"/>
+    <sheet name="Trial Balance" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="67">
   <si>
     <t>Asset Type</t>
   </si>
@@ -168,6 +170,81 @@
   </si>
   <si>
     <t>Frais courus - Fund-of-Funds</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Transaction Type</t>
+  </si>
+  <si>
+    <t>Credit account</t>
+  </si>
+  <si>
+    <t>Debit account</t>
+  </si>
+  <si>
+    <t>Subscription</t>
+  </si>
+  <si>
+    <t>Share Capital</t>
+  </si>
+  <si>
+    <t>Investor subscription</t>
+  </si>
+  <si>
+    <t>Dividend Income</t>
+  </si>
+  <si>
+    <t>Income (Dividends)</t>
+  </si>
+  <si>
+    <t>ASML dividend received</t>
+  </si>
+  <si>
+    <t>Daily management fee accrual</t>
+  </si>
+  <si>
+    <t>Fee Accrual</t>
+  </si>
+  <si>
+    <t>Management fees</t>
+  </si>
+  <si>
+    <t>Accrued fees</t>
+  </si>
+  <si>
+    <t>Accrued income</t>
+  </si>
+  <si>
+    <t>Interest Income</t>
+  </si>
+  <si>
+    <t>Interest Accrual</t>
+  </si>
+  <si>
+    <t>Bond interest accrual</t>
+  </si>
+  <si>
+    <t>Depositary fee payment</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Total Debit</t>
+  </si>
+  <si>
+    <t>Total Credit</t>
+  </si>
+  <si>
+    <t>Net Balance</t>
+  </si>
+  <si>
+    <t>Interest income</t>
   </si>
 </sst>
 </file>
@@ -257,7 +334,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -299,7 +376,10 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -842,10 +922,10 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="3" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="4">
@@ -1044,4 +1124,307 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FE4AC8B-72B8-4BE3-80AF-CFBD91888BFC}">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F2" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="4">
+        <v>16.02</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="4">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25C1313-92C4-4B45-AA8A-E858F6CE7DDC}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A2,'Transaction Journal'!F:F)</f>
+        <v>50800</v>
+      </c>
+      <c r="C2" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A2,'Transaction Journal'!F:F)</f>
+        <v>2500</v>
+      </c>
+      <c r="D2" s="3">
+        <f>+B2-C2</f>
+        <v>48300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A3,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A3,'Transaction Journal'!F:F)</f>
+        <v>50000</v>
+      </c>
+      <c r="D3" s="3">
+        <f t="shared" ref="D3:D9" si="0">+B3-C3</f>
+        <v>-50000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A4,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A4,'Transaction Journal'!F:F)</f>
+        <v>800</v>
+      </c>
+      <c r="D4" s="3">
+        <f t="shared" si="0"/>
+        <v>-800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A5,'Transaction Journal'!F:F)</f>
+        <v>16.02</v>
+      </c>
+      <c r="C5" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A5,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <f t="shared" si="0"/>
+        <v>16.02</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A6,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A6,'Transaction Journal'!F:F)</f>
+        <v>16.02</v>
+      </c>
+      <c r="D6" s="3">
+        <f t="shared" si="0"/>
+        <v>-16.02</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A7,'Transaction Journal'!F:F)</f>
+        <v>1150</v>
+      </c>
+      <c r="C7" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A7,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="3">
+        <f t="shared" si="0"/>
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A8,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A8,'Transaction Journal'!F:F)</f>
+        <v>1150</v>
+      </c>
+      <c r="D8" s="3">
+        <f t="shared" si="0"/>
+        <v>-1150</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="3">
+        <f>+SUMIF('Transaction Journal'!D:D,A9,'Transaction Journal'!F:F)</f>
+        <v>2500</v>
+      </c>
+      <c r="C9" s="3">
+        <f>+SUMIF('Transaction Journal'!E:E,A9,'Transaction Journal'!F:F)</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="24"/>
+      <c r="D10" s="25"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Traduction Excel en anglais
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{457DAB21-DA21-44E9-8C80-5FA1D9C46E54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DB9364-96AE-481A-9F2F-0AB4A7EC2D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
@@ -82,15 +82,9 @@
     <t>Receivable</t>
   </si>
   <si>
-    <t>Dividende ASML à recevoir</t>
-  </si>
-  <si>
     <t>Accrued Income</t>
   </si>
   <si>
-    <t>Intérêts courus (obligations)</t>
-  </si>
-  <si>
     <t>TOTAL ASSETS</t>
   </si>
   <si>
@@ -106,15 +100,6 @@
     <t>Accrued Fees</t>
   </si>
   <si>
-    <t>Facture dépositaire à payer</t>
-  </si>
-  <si>
-    <t>Frais de performance courus</t>
-  </si>
-  <si>
-    <t>Frais de gestion courus (daily)</t>
-  </si>
-  <si>
     <t>TOTAL LIABILITIES</t>
   </si>
   <si>
@@ -133,45 +118,12 @@
     <t>NAV per Share</t>
   </si>
   <si>
-    <t>Sous-fonds</t>
-  </si>
-  <si>
-    <t>Parts détenues</t>
-  </si>
-  <si>
-    <t>NAV par part du sous fonds</t>
-  </si>
-  <si>
-    <t>Frais du sous-fonds (annuel)</t>
-  </si>
-  <si>
-    <t>Sous-fonds A (obligations)</t>
-  </si>
-  <si>
-    <t>Sous-fonds B (actions US)</t>
-  </si>
-  <si>
-    <t>Sous-fonds C (actions émergentes)</t>
-  </si>
-  <si>
-    <t>Valeur de marché</t>
-  </si>
-  <si>
-    <t>Frais courus journaliers</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
     <t>Fund-of-Funds investment</t>
   </si>
   <si>
-    <t>Position consolidée 3 sous-fonds UCITS</t>
-  </si>
-  <si>
-    <t>Frais courus - Fund-of-Funds</t>
-  </si>
-  <si>
     <t>Date</t>
   </si>
   <si>
@@ -245,6 +197,54 @@
   </si>
   <si>
     <t>Interest income</t>
+  </si>
+  <si>
+    <t>ASML dividend receivable</t>
+  </si>
+  <si>
+    <t>Accrued bond interest</t>
+  </si>
+  <si>
+    <t>Consolidated position — 3 UCITS sub-funds</t>
+  </si>
+  <si>
+    <t>Depositary invoice payable</t>
+  </si>
+  <si>
+    <t>Accrued management fees (daily)</t>
+  </si>
+  <si>
+    <t>Accrued performance fees</t>
+  </si>
+  <si>
+    <t>Accrued fees — Fund-of-Funds</t>
+  </si>
+  <si>
+    <t>Sub-fund</t>
+  </si>
+  <si>
+    <t>Units held</t>
+  </si>
+  <si>
+    <t>Sub-fund NAV per unit</t>
+  </si>
+  <si>
+    <t>Annual sub-fund fee</t>
+  </si>
+  <si>
+    <t>Market value</t>
+  </si>
+  <si>
+    <t>Daily accrued fees</t>
+  </si>
+  <si>
+    <t>Sub-fund A (bonds)</t>
+  </si>
+  <si>
+    <t>Sub-fund B (US equities)</t>
+  </si>
+  <si>
+    <t>Sub-fund C (emerging market equities)</t>
   </si>
 </sst>
 </file>
@@ -334,7 +334,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -377,9 +377,8 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -804,7 +803,7 @@
       <c r="C5" s="5"/>
       <c r="D5" s="6"/>
       <c r="E5" s="21">
-        <v>85000</v>
+        <v>133300</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -812,7 +811,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>12</v>
+        <v>51</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="6"/>
@@ -822,10 +821,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="6"/>
@@ -835,10 +834,10 @@
     </row>
     <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="6"/>
@@ -849,14 +848,14 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="10">
         <f>+SUM(E2:E8)</f>
-        <v>584850</v>
+        <v>633150</v>
       </c>
     </row>
   </sheetData>
@@ -870,41 +869,40 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="C2" s="4">
-        <v>2500</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="C3" s="4">
-        <f>+(Assets!E9*Liabilities!F3)/365</f>
-        <v>16.023287671232875</v>
+        <v>16.02</v>
       </c>
       <c r="F3" s="7">
         <v>0.01</v>
@@ -912,10 +910,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>56</v>
       </c>
       <c r="C4" s="4">
         <v>1800</v>
@@ -923,10 +921,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="C5" s="4">
         <f>+'Fund-of-Funds'!F5</f>
@@ -935,12 +933,12 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="9">
         <f>+SUM(C2:C5)</f>
-        <v>4320.0260273972599</v>
+        <v>1820.0227397260273</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -962,46 +960,47 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B1" s="12">
         <f>+Assets!E9</f>
-        <v>584850</v>
+        <v>633150</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B2" s="12">
         <f>+Liabilities!C6</f>
-        <v>4320.0260273972599</v>
+        <v>1820.0227397260273</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B3" s="13">
         <f>+B1-B2</f>
-        <v>580529.97397260275</v>
+        <v>631329.977260274</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B4" s="14">
-        <v>4480</v>
+        <f>4480+385.86</f>
+        <v>4865.8599999999997</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B5" s="15">
         <f>+B3/B4</f>
-        <v>129.58258347602739</v>
+        <v>129.74684377690153</v>
       </c>
     </row>
   </sheetData>
@@ -1014,7 +1013,7 @@
   <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.77734375" customWidth="1"/>
     <col min="4" max="4" width="14.109375" customWidth="1"/>
@@ -1024,27 +1023,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="C1" s="19" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>32</v>
+        <v>61</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="B2" s="3">
         <v>500</v>
@@ -1066,7 +1065,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="B3" s="3">
         <v>300</v>
@@ -1087,8 +1086,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>35</v>
+      <c r="A4" s="25" t="s">
+        <v>66</v>
       </c>
       <c r="B4" s="3">
         <v>200</v>
@@ -1110,7 +1109,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <f>+SUM(E2:E4)</f>
@@ -1139,22 +1138,22 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1162,16 +1161,16 @@
         <v>46273</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="F2" s="4">
         <v>50000</v>
@@ -1182,16 +1181,16 @@
         <v>46273</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="F3" s="4">
         <v>800</v>
@@ -1202,16 +1201,16 @@
         <v>46273</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="F4" s="4">
         <v>16.02</v>
@@ -1222,16 +1221,16 @@
         <v>46273</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="F5" s="4">
         <v>1150</v>
@@ -1242,13 +1241,13 @@
         <v>46273</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>9</v>
@@ -1264,24 +1263,24 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25C1313-92C4-4B45-AA8A-E858F6CE7DDC}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
-        <v>62</v>
-      </c>
-      <c r="B1" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="26" t="s">
-        <v>65</v>
+      <c r="A1" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -1303,7 +1302,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B3" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A3,'Transaction Journal'!F:F)</f>
@@ -1320,7 +1319,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B4" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A4,'Transaction Journal'!F:F)</f>
@@ -1337,7 +1336,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B5" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A5,'Transaction Journal'!F:F)</f>
@@ -1354,7 +1353,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="B6" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A6,'Transaction Journal'!F:F)</f>
@@ -1371,7 +1370,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="B7" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A7,'Transaction Journal'!F:F)</f>
@@ -1388,7 +1387,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="B8" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A8,'Transaction Journal'!F:F)</f>
@@ -1405,7 +1404,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B9" s="3">
         <f>+SUMIF('Transaction Journal'!D:D,A9,'Transaction Journal'!F:F)</f>
@@ -1419,10 +1418,6 @@
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C10" s="24"/>
-      <c r="D10" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ajout module de réconciliation (fuzzy matching Python) - étape 4
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DB9364-96AE-481A-9F2F-0AB4A7EC2D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598A0E52-0998-4FAE-82BC-87CF9172C8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Fund-of-Funds" sheetId="4" r:id="rId4"/>
     <sheet name="Transaction Journal" sheetId="5" r:id="rId5"/>
     <sheet name="Trial Balance" sheetId="6" r:id="rId6"/>
+    <sheet name="Bank Statement" sheetId="7" r:id="rId7"/>
+    <sheet name="TJ_Export" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
   <si>
     <t>Asset Type</t>
   </si>
@@ -245,6 +247,12 @@
   </si>
   <si>
     <t>Sub-fund C (emerging market equities)</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Investor subscription received</t>
   </si>
 </sst>
 </file>
@@ -334,7 +342,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -378,7 +386,24 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers" xfId="1" builtinId="3"/>
@@ -1086,7 +1111,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="2" t="s">
         <v>66</v>
       </c>
       <c r="B4" s="3">
@@ -1422,4 +1447,132 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32E4AAA7-26C2-4E5D-831F-19D1505B49AD}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" style="1"/>
+    <col min="4" max="4" width="11.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="25">
+        <v>46273</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="27">
+        <v>50000</v>
+      </c>
+      <c r="D2" s="29">
+        <f>+C2</f>
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="25">
+        <v>46273</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="27">
+        <v>800</v>
+      </c>
+      <c r="D3" s="30">
+        <f>+D2+C3</f>
+        <v>50800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="25">
+        <v>46274</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="27">
+        <v>-2500</v>
+      </c>
+      <c r="D4" s="30">
+        <f>+D3+C4</f>
+        <v>48300</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF989E4D-4816-4BEB-9529-C34F0757E54E}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="4">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="4">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="23">
+        <v>46273</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="4">
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
README : liens cliquables, note de progression, skills demonstrated, ajout excel-skills
</commit_message>
<xml_diff>
--- a/nav/fund_alpha_nav_calculator.xlsx
+++ b/nav/fund_alpha_nav_calculator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devil\fund accounting roadmap\lux-fund-case-study\nav\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{598A0E52-0998-4FAE-82BC-87CF9172C8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41CE374-B61A-4C30-BF23-57A469F28C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="6" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{719DAA5C-B416-4958-BA3B-EFD9ABF611FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Trial Balance" sheetId="6" r:id="rId6"/>
     <sheet name="Bank Statement" sheetId="7" r:id="rId7"/>
     <sheet name="TJ_Export" sheetId="8" r:id="rId8"/>
+    <sheet name="XLOOKUP Practice" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="72">
   <si>
     <t>Asset Type</t>
   </si>
@@ -253,6 +254,15 @@
   </si>
   <si>
     <t>Investor subscription received</t>
+  </si>
+  <si>
+    <t>Bank Description</t>
+  </si>
+  <si>
+    <t>Bank Amount</t>
+  </si>
+  <si>
+    <t>Matched Journal Amount</t>
   </si>
 </sst>
 </file>
@@ -342,7 +352,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -403,6 +413,15 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1575,4 +1594,66 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A035158B-1048-420D-A8F4-49FEF493467A}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="B1" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="31" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="32">
+        <v>50000</v>
+      </c>
+      <c r="C2" s="31" t="str">
+        <f>+_xlfn.XLOOKUP(A2,'Transaction Journal'!C:C,'Transaction Journal'!F:F,"Non trouvé")</f>
+        <v>Non trouvé</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="32">
+        <v>800</v>
+      </c>
+      <c r="C3" s="31">
+        <f>+_xlfn.XLOOKUP(A3,'Transaction Journal'!C:C,'Transaction Journal'!F:F,"Non trouvé")</f>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="32">
+        <v>-2500</v>
+      </c>
+      <c r="C4" s="31">
+        <f>+_xlfn.XLOOKUP(A4,'Transaction Journal'!C:C,'Transaction Journal'!F:F,"Non trouvé")</f>
+        <v>2500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>